<commit_message>
RGBW board V0.3, creepage slots, mains-safety note on enclosure screws
RGBW load board moves to V0.3: 1032 ceramic fuse rated 250 V in place of
the 125 V Littelfuse 0154, and a pinout drawing for the first time. Both
load boards get slots that lengthen the creepage path from the mains copper
to the enclosure screws, and a 3.9 mm AC-to-LV clearance rule that checks
the air gap across those slots.

The screws only keep the required distance from the mains side when the
head rests on the plastic housing, never on the PCB itself. The Hardware
README and both load-board READMEs now say so.
</commit_message>
<xml_diff>
--- a/Hardware/DALI_Load_250W_DigitalLED/JLC_PCBA_BOM-DALI_LOAD_DigitalLED(V0.1).xlsx
+++ b/Hardware/DALI_Load_250W_DigitalLED/JLC_PCBA_BOM-DALI_LOAD_DigitalLED(V0.1).xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="111">
   <si>
     <t xml:space="preserve">Comment</t>
   </si>
@@ -311,6 +311,9 @@
     <t xml:space="preserve">C8598</t>
   </si>
   <si>
+    <t xml:space="preserve">C53035203</t>
+  </si>
+  <si>
     <t xml:space="preserve">C1002</t>
   </si>
   <si>
@@ -351,9 +354,6 @@
   </si>
   <si>
     <t xml:space="preserve">C970946</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C53035203</t>
   </si>
 </sst>
 </file>
@@ -840,7 +840,7 @@
         <v>1</v>
       </c>
       <c r="F10" t="s">
-        <v>110</v>
+        <v>96</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -860,7 +860,7 @@
         <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -897,7 +897,7 @@
         <v>1</v>
       </c>
       <c r="F13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -917,7 +917,7 @@
         <v>1</v>
       </c>
       <c r="F14" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -988,7 +988,7 @@
         <v>1</v>
       </c>
       <c r="F18" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -1008,7 +1008,7 @@
         <v>1</v>
       </c>
       <c r="F19" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -1028,7 +1028,7 @@
         <v>1</v>
       </c>
       <c r="F20" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -1048,7 +1048,7 @@
         <v>1</v>
       </c>
       <c r="F21" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -1068,7 +1068,7 @@
         <v>1</v>
       </c>
       <c r="F22" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -1088,7 +1088,7 @@
         <v>1</v>
       </c>
       <c r="F23" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -1108,7 +1108,7 @@
         <v>1</v>
       </c>
       <c r="F24" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -1128,7 +1128,7 @@
         <v>1</v>
       </c>
       <c r="F25" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -1148,7 +1148,7 @@
         <v>1</v>
       </c>
       <c r="F26" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -1168,7 +1168,7 @@
         <v>1</v>
       </c>
       <c r="F27" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -1188,7 +1188,7 @@
         <v>1</v>
       </c>
       <c r="F28" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>